<commit_message>
Add required column validation.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowbi-guard\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03DDCAE6-9141-430C-BCD1-23BF3756CF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C903459-E8D9-46B4-B7BB-55339EE271AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1455,7 +1455,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1467,11 +1467,69 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="14">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1485,20 +1543,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectsTable" displayName="ProjectsTable" ref="A1:L21" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectsTable" displayName="ProjectsTable" ref="A1:L21" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ProjectID"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ProjectName"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Department"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ProjectManager"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="City"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Program"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Priority"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="StartDate"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PlannedEndDate"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="BudgetSAR"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="AsOfDate"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="ProjectStatus"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ProjectID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ProjectName" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Department" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ProjectManager" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="City" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Program" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Priority" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="StartDate" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PlannedEndDate" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="BudgetSAR" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="AsOfDate" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="ProjectStatus" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1812,804 +1870,805 @@
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="12" width="22" customWidth="1"/>
+    <col min="1" max="12" width="22" style="8" customWidth="1"/>
+    <col min="13" max="16384" width="8.6640625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="34" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="10">
         <v>46027</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="10">
         <v>46207</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="11">
         <v>500000</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="10">
         <v>46312</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="10">
         <v>46038</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="10">
         <v>46263</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="11">
         <v>675000</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="10">
         <v>46312</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="10">
         <v>46049</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="10">
         <v>46319</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="11">
         <v>850000</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="10">
         <v>46312</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="24" customHeight="1">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="10">
         <v>46060</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="10">
         <v>46375</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="11">
         <v>1025000</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="10">
         <v>46312</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="24" customHeight="1">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="10">
         <v>46071</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="10">
         <v>46431</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="11">
         <v>1200000</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="10">
         <v>46312</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="24" customHeight="1">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="10">
         <v>46082</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="10">
         <v>46262</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="11">
         <v>1375000</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="10">
         <v>46312</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="10">
         <v>46093</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="10">
         <v>46318</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="11">
         <v>1550000</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="10">
         <v>46312</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="24" customHeight="1">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="10">
         <v>46104</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="10">
         <v>46374</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="11">
         <v>1725000</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="10">
         <v>46312</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="24" customHeight="1">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="10">
         <v>46115</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="10">
         <v>46430</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="11">
         <v>1900000</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="10">
         <v>46312</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="L10" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="24" customHeight="1">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="10">
         <v>46126</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="10">
         <v>46486</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="11">
         <v>2075000</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="10">
         <v>46312</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="24" customHeight="1">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="10">
         <v>46137</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="10">
         <v>46317</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="11">
         <v>2250000</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="10">
         <v>46312</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="L12" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="24" customHeight="1">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="10">
         <v>46148</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="10">
         <v>46373</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="11">
         <v>2425000</v>
       </c>
-      <c r="K13" s="3">
+      <c r="K13" s="10">
         <v>46312</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="L13" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="24" customHeight="1">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="10">
         <v>46159</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="10">
         <v>46429</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="11">
         <v>2600000</v>
       </c>
-      <c r="K14" s="3">
+      <c r="K14" s="10">
         <v>46312</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="L14" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="24" customHeight="1">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="10">
         <v>46170</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="10">
         <v>46485</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="11">
         <v>2775000</v>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="10">
         <v>46312</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="L15" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="24" customHeight="1">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="10">
         <v>46181</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="10">
         <v>46541</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="11">
         <v>2950000</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="10">
         <v>46312</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="L16" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="24" customHeight="1">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="10">
         <v>46192</v>
       </c>
-      <c r="I17" s="3">
+      <c r="I17" s="10">
         <v>46372</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="11">
         <v>3125000</v>
       </c>
-      <c r="K17" s="3">
+      <c r="K17" s="10">
         <v>46312</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="L17" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="24" customHeight="1">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="10">
         <v>46203</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18" s="10">
         <v>46428</v>
       </c>
-      <c r="J18" s="4">
+      <c r="J18" s="11">
         <v>3300000</v>
       </c>
-      <c r="K18" s="3">
+      <c r="K18" s="10">
         <v>46312</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="L18" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="24" customHeight="1">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="10">
         <v>46214</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="10">
         <v>46484</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19" s="11">
         <v>3475000</v>
       </c>
-      <c r="K19" s="3">
+      <c r="K19" s="10">
         <v>46312</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="L19" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="24" customHeight="1">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="10">
         <v>46225</v>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" s="10">
         <v>46540</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J20" s="11">
         <v>3650000</v>
       </c>
-      <c r="K20" s="3">
+      <c r="K20" s="10">
         <v>46312</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="L20" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="24" customHeight="1">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G21" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="10">
         <v>46236</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="10">
         <v>46596</v>
       </c>
-      <c r="J21" s="4">
+      <c r="J21" s="11">
         <v>3825000</v>
       </c>
-      <c r="K21" s="3">
+      <c r="K21" s="10">
         <v>46312</v>
       </c>
-      <c r="L21" s="1" t="s">
+      <c r="L21" s="9" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>